<commit_message>
Add files via upload
</commit_message>
<xml_diff>
--- a/Sprint1 using the excel.xml.xlsx
+++ b/Sprint1 using the excel.xml.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91812\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aspire 5 15\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB4C426E-D65E-4D59-B961-891BBCE5A19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BBE203-006B-4E2E-8FF5-D786967C0C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{B652266E-C761-44B3-942B-E4E0463E8619}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{B652266E-C761-44B3-942B-E4E0463E8619}"/>
   </bookViews>
   <sheets>
     <sheet name="Placement_RawData_Full_Class " sheetId="1" r:id="rId1"/>
@@ -1071,6 +1071,30 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -1102,6 +1126,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-4CC4-4082-9602-D80D4E7FE521}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -1115,6 +1144,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-4CC4-4082-9602-D80D4E7FE521}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -3203,6 +3237,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -3247,6 +3290,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -4502,7 +4554,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1D53-40BB-ABDE-6ECD6F703F8F}"/>
+              <c16:uniqueId val="{00000000-587E-4542-A927-C83768CF5AAD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6288,6 +6340,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -6332,6 +6393,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -7597,7 +7667,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4FF2-4627-9E13-32D29371656B}"/>
+              <c16:uniqueId val="{00000001-0237-4B0F-84DA-E38A23C4728E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -13655,9 +13725,6 @@
             </a:rPr>
             <a:t>Placement Student </a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
           <a:endParaRPr lang="en-IN" sz="1100"/>
         </a:p>
         <a:p>
@@ -14332,8 +14399,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>50801</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="15" name="gender">
@@ -14356,7 +14423,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -14410,8 +14477,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>44450</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="16" name="degree_t">
@@ -14434,7 +14501,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -14488,8 +14555,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>38101</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="17" name="specialisation">
@@ -14512,7 +14579,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -14566,8 +14633,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>31751</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="18" name="workex">
@@ -14590,7 +14657,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -14644,8 +14711,8 @@
       <xdr:row>33</xdr:row>
       <xdr:rowOff>38101</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="19" name="status">
@@ -14668,7 +14735,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -18449,240 +18516,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DFEDC587-2D02-49CE-A089-DA61171EB606}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
-  <location ref="J3:M5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colFields count="1">
-    <field x="13"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of status" fld="13" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="8" format="6" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="8" format="7" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7038C755-7E3D-4855-85E2-2008BCD94654}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
-  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="15">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="3">
-        <item x="1"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="13"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of status" fld="13" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="5">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="12" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F788E398-8292-4538-9617-50206FB46560}" name="PivotTable6" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12">
   <location ref="J53:K56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="15">
@@ -18778,7 +18611,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79FB3E5E-1A94-4FBB-AE2F-3703BDC76A79}" name="PivotTable5" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="A52:D57" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
@@ -18925,7 +18758,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E72D361F-97A6-4715-A345-594B3A6CFA21}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="J28:M32" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
@@ -19068,7 +18901,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{313D1DEC-5C03-4173-9328-944E74FBD87B}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="A27:D31" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="15">
@@ -19169,6 +19002,264 @@
       </pivotArea>
     </chartFormat>
     <chartFormat chart="9" format="13" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DFEDC587-2D02-49CE-A089-DA61171EB606}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+  <location ref="J3:M5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="13"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of status" fld="13" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="6" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="8" format="7" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7038C755-7E3D-4855-85E2-2008BCD94654}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="15">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="13"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of status" fld="13" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -19606,14 +19697,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27B0B069-5269-43E3-822E-85043C7AD20E}">
   <dimension ref="A1:O219"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="7.81640625" customWidth="1"/>
-    <col min="7" max="7" width="7.81640625" customWidth="1"/>
-    <col min="9" max="9" width="7.1796875" customWidth="1"/>
+    <col min="2" max="2" width="7.77734375" customWidth="1"/>
+    <col min="7" max="7" width="7.77734375" customWidth="1"/>
+    <col min="9" max="9" width="7.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -19660,7 +19751,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -19707,7 +19798,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -19754,7 +19845,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -19801,7 +19892,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -19848,7 +19939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -19895,7 +19986,7 @@
         <v>425000</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -19942,7 +20033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -19989,7 +20080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -20036,7 +20127,7 @@
         <v>252000</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -20083,7 +20174,7 @@
         <v>231000</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -20130,7 +20221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -20177,7 +20268,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -20224,7 +20315,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -20271,7 +20362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -20318,7 +20409,7 @@
         <v>218000</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -20365,7 +20456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -20412,7 +20503,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -20459,7 +20550,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -20506,7 +20597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -20553,7 +20644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -20600,7 +20691,7 @@
         <v>236000</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -20647,7 +20738,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
@@ -20694,7 +20785,7 @@
         <v>393000</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -20741,7 +20832,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -20788,7 +20879,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -20835,7 +20926,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -20882,7 +20973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
@@ -20929,7 +21020,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -20976,7 +21067,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -21023,7 +21114,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -21070,7 +21161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
@@ -21117,7 +21208,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
@@ -21164,7 +21255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
@@ -21211,7 +21302,7 @@
         <v>278000</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -21258,7 +21349,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
@@ -21305,7 +21396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -21352,7 +21443,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
@@ -21399,7 +21490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>38</v>
       </c>
@@ -21446,7 +21537,7 @@
         <v>320000</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>39</v>
       </c>
@@ -21493,7 +21584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -21540,7 +21631,7 @@
         <v>411000</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>41</v>
       </c>
@@ -21587,7 +21678,7 @@
         <v>287000</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>42</v>
       </c>
@@ -21634,7 +21725,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -21681,7 +21772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -21728,7 +21819,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45</v>
       </c>
@@ -21775,7 +21866,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>46</v>
       </c>
@@ -21822,7 +21913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>47</v>
       </c>
@@ -21869,7 +21960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>48</v>
       </c>
@@ -21916,7 +22007,7 @@
         <v>204000</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>49</v>
       </c>
@@ -21963,7 +22054,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>50</v>
       </c>
@@ -22004,7 +22095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>50</v>
       </c>
@@ -22051,7 +22142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>51</v>
       </c>
@@ -22098,7 +22189,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>52</v>
       </c>
@@ -22145,7 +22236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>53</v>
       </c>
@@ -22192,7 +22283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>54</v>
       </c>
@@ -22239,7 +22330,7 @@
         <v>450000</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>55</v>
       </c>
@@ -22286,7 +22377,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>56</v>
       </c>
@@ -22333,7 +22424,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>57</v>
       </c>
@@ -22380,7 +22471,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>58</v>
       </c>
@@ -22427,7 +22518,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>59</v>
       </c>
@@ -22474,7 +22565,7 @@
         <v>268000</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>60</v>
       </c>
@@ -22521,7 +22612,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>61</v>
       </c>
@@ -22568,7 +22659,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>62</v>
       </c>
@@ -22615,7 +22706,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>63</v>
       </c>
@@ -22662,7 +22753,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>64</v>
       </c>
@@ -22709,7 +22800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>65</v>
       </c>
@@ -22756,7 +22847,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>66</v>
       </c>
@@ -22803,7 +22894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>67</v>
       </c>
@@ -22850,7 +22941,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>68</v>
       </c>
@@ -22897,7 +22988,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>69</v>
       </c>
@@ -22944,7 +23035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>70</v>
       </c>
@@ -22991,7 +23082,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>71</v>
       </c>
@@ -23038,7 +23129,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>72</v>
       </c>
@@ -23085,7 +23176,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>73</v>
       </c>
@@ -23132,7 +23223,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>74</v>
       </c>
@@ -23179,7 +23270,7 @@
         <v>218000</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>75</v>
       </c>
@@ -23226,7 +23317,7 @@
         <v>336000</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>76</v>
       </c>
@@ -23273,7 +23364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>77</v>
       </c>
@@ -23320,7 +23411,7 @@
         <v>230000</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>78</v>
       </c>
@@ -23367,7 +23458,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>79</v>
       </c>
@@ -23414,7 +23505,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>80</v>
       </c>
@@ -23461,7 +23552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>81</v>
       </c>
@@ -23508,7 +23599,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>82</v>
       </c>
@@ -23555,7 +23646,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>83</v>
       </c>
@@ -23602,7 +23693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>84</v>
       </c>
@@ -23649,7 +23740,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>85</v>
       </c>
@@ -23696,7 +23787,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>86</v>
       </c>
@@ -23743,7 +23834,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>87</v>
       </c>
@@ -23790,7 +23881,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>88</v>
       </c>
@@ -23837,7 +23928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>89</v>
       </c>
@@ -23884,7 +23975,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>89</v>
       </c>
@@ -23931,7 +24022,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>90</v>
       </c>
@@ -23978,7 +24069,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>91</v>
       </c>
@@ -24025,7 +24116,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>92</v>
       </c>
@@ -24072,7 +24163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>93</v>
       </c>
@@ -24119,7 +24210,7 @@
         <v>230000</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>94</v>
       </c>
@@ -24166,7 +24257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>95</v>
       </c>
@@ -24213,7 +24304,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>96</v>
       </c>
@@ -24260,7 +24351,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>97</v>
       </c>
@@ -24307,7 +24398,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>98</v>
       </c>
@@ -24354,7 +24445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>99</v>
       </c>
@@ -24401,7 +24492,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>100</v>
       </c>
@@ -24448,7 +24539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>101</v>
       </c>
@@ -24495,7 +24586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>102</v>
       </c>
@@ -24542,7 +24633,7 @@
         <v>380000</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>103</v>
       </c>
@@ -24589,7 +24680,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>104</v>
       </c>
@@ -24636,7 +24727,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>105</v>
       </c>
@@ -24683,7 +24774,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>106</v>
       </c>
@@ -24730,7 +24821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>107</v>
       </c>
@@ -24777,7 +24868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>108</v>
       </c>
@@ -24824,7 +24915,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>109</v>
       </c>
@@ -24871,7 +24962,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>110</v>
       </c>
@@ -24918,7 +25009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>111</v>
       </c>
@@ -24965,7 +25056,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>112</v>
       </c>
@@ -25012,7 +25103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>113</v>
       </c>
@@ -25059,7 +25150,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>114</v>
       </c>
@@ -25106,7 +25197,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>115</v>
       </c>
@@ -25153,7 +25244,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>116</v>
       </c>
@@ -25200,7 +25291,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>117</v>
       </c>
@@ -25247,7 +25338,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>118</v>
       </c>
@@ -25294,7 +25385,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>119</v>
       </c>
@@ -25341,7 +25432,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>120</v>
       </c>
@@ -25388,7 +25479,7 @@
         <v>940000</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>121</v>
       </c>
@@ -25435,7 +25526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>122</v>
       </c>
@@ -25482,7 +25573,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>123</v>
       </c>
@@ -25529,7 +25620,7 @@
         <v>236000</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>124</v>
       </c>
@@ -25576,7 +25667,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>125</v>
       </c>
@@ -25623,7 +25714,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>126</v>
       </c>
@@ -25670,7 +25761,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>127</v>
       </c>
@@ -25717,7 +25808,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>128</v>
       </c>
@@ -25764,7 +25855,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>129</v>
       </c>
@@ -25811,7 +25902,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>130</v>
       </c>
@@ -25858,7 +25949,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>131</v>
       </c>
@@ -25905,7 +25996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>132</v>
       </c>
@@ -25952,7 +26043,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>133</v>
       </c>
@@ -25999,7 +26090,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>134</v>
       </c>
@@ -26046,7 +26137,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>135</v>
       </c>
@@ -26093,7 +26184,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>136</v>
       </c>
@@ -26140,7 +26231,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>137</v>
       </c>
@@ -26187,7 +26278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>138</v>
       </c>
@@ -26234,7 +26325,7 @@
         <v>225000</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>139</v>
       </c>
@@ -26281,7 +26372,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>140</v>
       </c>
@@ -26328,7 +26419,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>141</v>
       </c>
@@ -26375,7 +26466,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>142</v>
       </c>
@@ -26422,7 +26513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>143</v>
       </c>
@@ -26469,7 +26560,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>144</v>
       </c>
@@ -26516,7 +26607,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>145</v>
       </c>
@@ -26563,7 +26654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>146</v>
       </c>
@@ -26610,7 +26701,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>147</v>
       </c>
@@ -26657,7 +26748,7 @@
         <v>233000</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>148</v>
       </c>
@@ -26704,7 +26795,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>149</v>
       </c>
@@ -26751,7 +26842,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>150</v>
       </c>
@@ -26798,7 +26889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>151</v>
       </c>
@@ -26845,7 +26936,7 @@
         <v>690000</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>152</v>
       </c>
@@ -26892,7 +26983,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>153</v>
       </c>
@@ -26939,7 +27030,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>154</v>
       </c>
@@ -26986,7 +27077,7 @@
         <v>340000</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>155</v>
       </c>
@@ -27033,7 +27124,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>156</v>
       </c>
@@ -27080,7 +27171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>157</v>
       </c>
@@ -27127,7 +27218,7 @@
         <v>255000</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>158</v>
       </c>
@@ -27174,7 +27265,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>159</v>
       </c>
@@ -27221,7 +27312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>160</v>
       </c>
@@ -27268,7 +27359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>161</v>
       </c>
@@ -27315,7 +27406,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>162</v>
       </c>
@@ -27362,7 +27453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>163</v>
       </c>
@@ -27409,7 +27500,7 @@
         <v>285000</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>164</v>
       </c>
@@ -27456,7 +27547,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>165</v>
       </c>
@@ -27503,7 +27594,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>166</v>
       </c>
@@ -27550,7 +27641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>167</v>
       </c>
@@ -27597,7 +27688,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>168</v>
       </c>
@@ -27644,7 +27735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>169</v>
       </c>
@@ -27691,7 +27782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>170</v>
       </c>
@@ -27738,7 +27829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>171</v>
       </c>
@@ -27785,7 +27876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>172</v>
       </c>
@@ -27832,7 +27923,7 @@
         <v>290000</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>173</v>
       </c>
@@ -27879,7 +27970,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>174</v>
       </c>
@@ -27926,7 +28017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>175</v>
       </c>
@@ -27973,7 +28064,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>176</v>
       </c>
@@ -28020,7 +28111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>177</v>
       </c>
@@ -28067,7 +28158,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>178</v>
       </c>
@@ -28114,7 +28205,7 @@
         <v>650000</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>179</v>
       </c>
@@ -28161,7 +28252,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>180</v>
       </c>
@@ -28208,7 +28299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>181</v>
       </c>
@@ -28255,7 +28346,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>182</v>
       </c>
@@ -28302,7 +28393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>183</v>
       </c>
@@ -28349,7 +28440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>184</v>
       </c>
@@ -28396,7 +28487,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>185</v>
       </c>
@@ -28443,7 +28534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>186</v>
       </c>
@@ -28490,7 +28581,7 @@
         <v>252000</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>187</v>
       </c>
@@ -28537,7 +28628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>188</v>
       </c>
@@ -28584,7 +28675,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>189</v>
       </c>
@@ -28631,7 +28722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>190</v>
       </c>
@@ -28678,7 +28769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>191</v>
       </c>
@@ -28725,7 +28816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>192</v>
       </c>
@@ -28772,7 +28863,7 @@
         <v>264000</v>
       </c>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>193</v>
       </c>
@@ -28819,7 +28910,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>194</v>
       </c>
@@ -28866,7 +28957,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>195</v>
       </c>
@@ -28913,7 +29004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>196</v>
       </c>
@@ -28960,7 +29051,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>197</v>
       </c>
@@ -29007,7 +29098,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>198</v>
       </c>
@@ -29054,7 +29145,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>199</v>
       </c>
@@ -29101,7 +29192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>200</v>
       </c>
@@ -29148,7 +29239,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>201</v>
       </c>
@@ -29195,7 +29286,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>202</v>
       </c>
@@ -29242,7 +29333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>203</v>
       </c>
@@ -29289,7 +29380,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>204</v>
       </c>
@@ -29336,7 +29427,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>205</v>
       </c>
@@ -29383,7 +29474,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>206</v>
       </c>
@@ -29430,7 +29521,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>207</v>
       </c>
@@ -29477,7 +29568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>208</v>
       </c>
@@ -29524,7 +29615,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>209</v>
       </c>
@@ -29571,7 +29662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>210</v>
       </c>
@@ -29618,7 +29709,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>211</v>
       </c>
@@ -29665,7 +29756,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>212</v>
       </c>
@@ -29712,7 +29803,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>213</v>
       </c>
@@ -29759,7 +29850,7 @@
         <v>295000</v>
       </c>
     </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>214</v>
       </c>
@@ -29806,7 +29897,7 @@
         <v>204000</v>
       </c>
     </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>215</v>
       </c>
@@ -29861,21 +29952,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CF27F7E-AB0E-4DB4-BB64-0D5FF33599C2}">
   <dimension ref="A1:O216"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="8.90625" style="1"/>
-    <col min="7" max="7" width="12.453125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="13.81640625" style="1" customWidth="1"/>
+    <col min="1" max="6" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="13.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="9" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" style="1" customWidth="1"/>
-    <col min="12" max="12" width="14.453125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="8.90625" style="1"/>
+    <col min="11" max="11" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.44140625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="8.88671875" style="1"/>
     <col min="14" max="14" width="13" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.90625" style="1"/>
+    <col min="15" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -29922,7 +30013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -29969,7 +30060,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -30016,7 +30107,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="6">
         <v>3</v>
       </c>
@@ -30063,7 +30154,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="6">
         <v>4</v>
       </c>
@@ -30110,7 +30201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -30157,7 +30248,7 @@
         <v>425000</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>6</v>
       </c>
@@ -30204,7 +30295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="6">
         <v>7</v>
       </c>
@@ -30251,7 +30342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>8</v>
       </c>
@@ -30298,7 +30389,7 @@
         <v>252000</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="6">
         <v>9</v>
       </c>
@@ -30345,7 +30436,7 @@
         <v>231000</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>10</v>
       </c>
@@ -30392,7 +30483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>11</v>
       </c>
@@ -30439,7 +30530,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>12</v>
       </c>
@@ -30486,7 +30577,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="6">
         <v>13</v>
       </c>
@@ -30533,7 +30624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>14</v>
       </c>
@@ -30580,7 +30671,7 @@
         <v>218000</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="6">
         <v>15</v>
       </c>
@@ -30627,7 +30718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>16</v>
       </c>
@@ -30674,7 +30765,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -30721,7 +30812,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>18</v>
       </c>
@@ -30768,7 +30859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="6">
         <v>19</v>
       </c>
@@ -30815,7 +30906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>20</v>
       </c>
@@ -30862,7 +30953,7 @@
         <v>236000</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
         <v>21</v>
       </c>
@@ -30909,7 +31000,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>22</v>
       </c>
@@ -30956,7 +31047,7 @@
         <v>393000</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
         <v>23</v>
       </c>
@@ -31003,7 +31094,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>24</v>
       </c>
@@ -31050,7 +31141,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="6">
         <v>25</v>
       </c>
@@ -31097,7 +31188,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>26</v>
       </c>
@@ -31144,7 +31235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="6">
         <v>27</v>
       </c>
@@ -31191,7 +31282,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>28</v>
       </c>
@@ -31238,7 +31329,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="6">
         <v>29</v>
       </c>
@@ -31285,7 +31376,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>30</v>
       </c>
@@ -31332,7 +31423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="6">
         <v>31</v>
       </c>
@@ -31379,7 +31470,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>32</v>
       </c>
@@ -31426,7 +31517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="6">
         <v>33</v>
       </c>
@@ -31473,7 +31564,7 @@
         <v>278000</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>34</v>
       </c>
@@ -31520,7 +31611,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="6">
         <v>35</v>
       </c>
@@ -31567,7 +31658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>36</v>
       </c>
@@ -31614,7 +31705,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="6">
         <v>37</v>
       </c>
@@ -31661,7 +31752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>38</v>
       </c>
@@ -31708,7 +31799,7 @@
         <v>320000</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="6">
         <v>39</v>
       </c>
@@ -31755,7 +31846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>40</v>
       </c>
@@ -31802,7 +31893,7 @@
         <v>411000</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="6">
         <v>41</v>
       </c>
@@ -31849,7 +31940,7 @@
         <v>287000</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>42</v>
       </c>
@@ -31896,7 +31987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="6">
         <v>43</v>
       </c>
@@ -31943,7 +32034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="6">
         <v>44</v>
       </c>
@@ -31990,7 +32081,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="6">
         <v>45</v>
       </c>
@@ -32037,7 +32128,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="6">
         <v>46</v>
       </c>
@@ -32084,7 +32175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="6">
         <v>47</v>
       </c>
@@ -32131,7 +32222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="6">
         <v>48</v>
       </c>
@@ -32178,7 +32269,7 @@
         <v>204000</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="6">
         <v>49</v>
       </c>
@@ -32225,7 +32316,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="6">
         <v>50</v>
       </c>
@@ -32272,7 +32363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="6">
         <v>51</v>
       </c>
@@ -32319,7 +32410,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="6">
         <v>52</v>
       </c>
@@ -32366,7 +32457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="6">
         <v>53</v>
       </c>
@@ -32413,7 +32504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="6">
         <v>54</v>
       </c>
@@ -32460,7 +32551,7 @@
         <v>450000</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="6">
         <v>55</v>
       </c>
@@ -32507,7 +32598,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="6">
         <v>56</v>
       </c>
@@ -32554,7 +32645,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="6">
         <v>57</v>
       </c>
@@ -32601,7 +32692,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="6">
         <v>58</v>
       </c>
@@ -32648,7 +32739,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="6">
         <v>59</v>
       </c>
@@ -32695,7 +32786,7 @@
         <v>268000</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="6">
         <v>60</v>
       </c>
@@ -32742,7 +32833,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="6">
         <v>61</v>
       </c>
@@ -32789,7 +32880,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="6">
         <v>62</v>
       </c>
@@ -32836,7 +32927,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="6">
         <v>63</v>
       </c>
@@ -32883,7 +32974,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="6">
         <v>64</v>
       </c>
@@ -32930,7 +33021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="6">
         <v>65</v>
       </c>
@@ -32977,7 +33068,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="6">
         <v>66</v>
       </c>
@@ -33024,7 +33115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="6">
         <v>67</v>
       </c>
@@ -33071,7 +33162,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="6">
         <v>68</v>
       </c>
@@ -33118,7 +33209,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="6">
         <v>69</v>
       </c>
@@ -33165,7 +33256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="6">
         <v>70</v>
       </c>
@@ -33212,7 +33303,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="6">
         <v>71</v>
       </c>
@@ -33259,7 +33350,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="6">
         <v>72</v>
       </c>
@@ -33306,7 +33397,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="6">
         <v>73</v>
       </c>
@@ -33353,7 +33444,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75" s="6">
         <v>74</v>
       </c>
@@ -33400,7 +33491,7 @@
         <v>218000</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76" s="6">
         <v>75</v>
       </c>
@@ -33447,7 +33538,7 @@
         <v>336000</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77" s="6">
         <v>76</v>
       </c>
@@ -33494,7 +33585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="6">
         <v>77</v>
       </c>
@@ -33541,7 +33632,7 @@
         <v>230000</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79" s="6">
         <v>78</v>
       </c>
@@ -33588,7 +33679,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="6">
         <v>79</v>
       </c>
@@ -33635,7 +33726,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81" s="6">
         <v>80</v>
       </c>
@@ -33682,7 +33773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82" s="6">
         <v>81</v>
       </c>
@@ -33729,7 +33820,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83" s="6">
         <v>82</v>
       </c>
@@ -33776,7 +33867,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" s="6">
         <v>83</v>
       </c>
@@ -33823,7 +33914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" s="6">
         <v>84</v>
       </c>
@@ -33870,7 +33961,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" s="6">
         <v>85</v>
       </c>
@@ -33917,7 +34008,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87" s="6">
         <v>86</v>
       </c>
@@ -33964,7 +34055,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" s="6">
         <v>87</v>
       </c>
@@ -34011,7 +34102,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" s="6">
         <v>88</v>
       </c>
@@ -34058,7 +34149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90" s="6">
         <v>89</v>
       </c>
@@ -34105,7 +34196,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91" s="6">
         <v>90</v>
       </c>
@@ -34152,7 +34243,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92" s="6">
         <v>91</v>
       </c>
@@ -34199,7 +34290,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93" s="6">
         <v>92</v>
       </c>
@@ -34246,7 +34337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94" s="6">
         <v>93</v>
       </c>
@@ -34293,7 +34384,7 @@
         <v>230000</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95" s="6">
         <v>94</v>
       </c>
@@ -34340,7 +34431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96" s="6">
         <v>95</v>
       </c>
@@ -34387,7 +34478,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97" s="6">
         <v>96</v>
       </c>
@@ -34434,7 +34525,7 @@
         <v>420000</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98" s="6">
         <v>97</v>
       </c>
@@ -34481,7 +34572,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" s="6">
         <v>98</v>
       </c>
@@ -34528,7 +34619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" s="6">
         <v>99</v>
       </c>
@@ -34575,7 +34666,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" s="6">
         <v>100</v>
       </c>
@@ -34622,7 +34713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" s="6">
         <v>101</v>
       </c>
@@ -34669,7 +34760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" s="6">
         <v>102</v>
       </c>
@@ -34716,7 +34807,7 @@
         <v>380000</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" s="6">
         <v>103</v>
       </c>
@@ -34763,7 +34854,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" s="6">
         <v>104</v>
       </c>
@@ -34810,7 +34901,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="6">
         <v>105</v>
       </c>
@@ -34857,7 +34948,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="6">
         <v>106</v>
       </c>
@@ -34904,7 +34995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="6">
         <v>107</v>
       </c>
@@ -34951,7 +35042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="6">
         <v>108</v>
       </c>
@@ -34998,7 +35089,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="6">
         <v>109</v>
       </c>
@@ -35045,7 +35136,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="6">
         <v>110</v>
       </c>
@@ -35092,7 +35183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="6">
         <v>111</v>
       </c>
@@ -35139,7 +35230,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" s="6">
         <v>112</v>
       </c>
@@ -35186,7 +35277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" s="6">
         <v>113</v>
       </c>
@@ -35233,7 +35324,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" s="6">
         <v>114</v>
       </c>
@@ -35280,7 +35371,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" s="6">
         <v>115</v>
       </c>
@@ -35327,7 +35418,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" s="6">
         <v>116</v>
       </c>
@@ -35374,7 +35465,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" s="6">
         <v>117</v>
       </c>
@@ -35421,7 +35512,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" s="6">
         <v>118</v>
       </c>
@@ -35468,7 +35559,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120" s="6">
         <v>119</v>
       </c>
@@ -35515,7 +35606,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121" s="6">
         <v>120</v>
       </c>
@@ -35562,7 +35653,7 @@
         <v>940000</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122" s="6">
         <v>121</v>
       </c>
@@ -35609,7 +35700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123" s="6">
         <v>122</v>
       </c>
@@ -35656,7 +35747,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" s="6">
         <v>123</v>
       </c>
@@ -35703,7 +35794,7 @@
         <v>236000</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" s="6">
         <v>124</v>
       </c>
@@ -35750,7 +35841,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A126" s="6">
         <v>125</v>
       </c>
@@ -35797,7 +35888,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A127" s="6">
         <v>126</v>
       </c>
@@ -35844,7 +35935,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A128" s="6">
         <v>127</v>
       </c>
@@ -35891,7 +35982,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A129" s="6">
         <v>128</v>
       </c>
@@ -35938,7 +36029,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A130" s="6">
         <v>129</v>
       </c>
@@ -35985,7 +36076,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A131" s="6">
         <v>130</v>
       </c>
@@ -36032,7 +36123,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A132" s="6">
         <v>131</v>
       </c>
@@ -36079,7 +36170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A133" s="6">
         <v>132</v>
       </c>
@@ -36126,7 +36217,7 @@
         <v>360000</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A134" s="6">
         <v>133</v>
       </c>
@@ -36173,7 +36264,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A135" s="6">
         <v>134</v>
       </c>
@@ -36220,7 +36311,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A136" s="6">
         <v>135</v>
       </c>
@@ -36267,7 +36358,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A137" s="6">
         <v>136</v>
       </c>
@@ -36314,7 +36405,7 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A138" s="6">
         <v>137</v>
       </c>
@@ -36361,7 +36452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A139" s="6">
         <v>138</v>
       </c>
@@ -36408,7 +36499,7 @@
         <v>225000</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A140" s="6">
         <v>139</v>
       </c>
@@ -36455,7 +36546,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A141" s="6">
         <v>140</v>
       </c>
@@ -36502,7 +36593,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A142" s="6">
         <v>141</v>
       </c>
@@ -36549,7 +36640,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A143" s="6">
         <v>142</v>
       </c>
@@ -36596,7 +36687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A144" s="6">
         <v>143</v>
       </c>
@@ -36643,7 +36734,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A145" s="6">
         <v>144</v>
       </c>
@@ -36690,7 +36781,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A146" s="6">
         <v>145</v>
       </c>
@@ -36737,7 +36828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A147" s="6">
         <v>146</v>
       </c>
@@ -36784,7 +36875,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A148" s="6">
         <v>147</v>
       </c>
@@ -36831,7 +36922,7 @@
         <v>233000</v>
       </c>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A149" s="6">
         <v>148</v>
       </c>
@@ -36878,7 +36969,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A150" s="6">
         <v>149</v>
       </c>
@@ -36925,7 +37016,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A151" s="6">
         <v>150</v>
       </c>
@@ -36972,7 +37063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A152" s="6">
         <v>151</v>
       </c>
@@ -37019,7 +37110,7 @@
         <v>690000</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A153" s="6">
         <v>152</v>
       </c>
@@ -37066,7 +37157,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A154" s="6">
         <v>153</v>
       </c>
@@ -37113,7 +37204,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A155" s="6">
         <v>154</v>
       </c>
@@ -37160,7 +37251,7 @@
         <v>340000</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A156" s="6">
         <v>155</v>
       </c>
@@ -37207,7 +37298,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A157" s="6">
         <v>156</v>
       </c>
@@ -37254,7 +37345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A158" s="6">
         <v>157</v>
       </c>
@@ -37301,7 +37392,7 @@
         <v>255000</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A159" s="6">
         <v>158</v>
       </c>
@@ -37348,7 +37439,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A160" s="6">
         <v>159</v>
       </c>
@@ -37395,7 +37486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A161" s="6">
         <v>160</v>
       </c>
@@ -37442,7 +37533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A162" s="6">
         <v>161</v>
       </c>
@@ -37489,7 +37580,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A163" s="6">
         <v>162</v>
       </c>
@@ -37536,7 +37627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A164" s="6">
         <v>163</v>
       </c>
@@ -37583,7 +37674,7 @@
         <v>285000</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A165" s="6">
         <v>164</v>
       </c>
@@ -37630,7 +37721,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A166" s="6">
         <v>165</v>
       </c>
@@ -37677,7 +37768,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A167" s="6">
         <v>166</v>
       </c>
@@ -37724,7 +37815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A168" s="6">
         <v>167</v>
       </c>
@@ -37771,7 +37862,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A169" s="6">
         <v>168</v>
       </c>
@@ -37818,7 +37909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A170" s="6">
         <v>169</v>
       </c>
@@ -37865,7 +37956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A171" s="6">
         <v>170</v>
       </c>
@@ -37912,7 +38003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A172" s="6">
         <v>171</v>
       </c>
@@ -37959,7 +38050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A173" s="6">
         <v>172</v>
       </c>
@@ -38006,7 +38097,7 @@
         <v>290000</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A174" s="6">
         <v>173</v>
       </c>
@@ -38053,7 +38144,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A175" s="6">
         <v>174</v>
       </c>
@@ -38100,7 +38191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A176" s="6">
         <v>175</v>
       </c>
@@ -38147,7 +38238,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A177" s="6">
         <v>176</v>
       </c>
@@ -38194,7 +38285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A178" s="6">
         <v>177</v>
       </c>
@@ -38241,7 +38332,7 @@
         <v>220000</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A179" s="6">
         <v>178</v>
       </c>
@@ -38288,7 +38379,7 @@
         <v>650000</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A180" s="6">
         <v>179</v>
       </c>
@@ -38335,7 +38426,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A181" s="6">
         <v>180</v>
       </c>
@@ -38382,7 +38473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A182" s="6">
         <v>181</v>
       </c>
@@ -38429,7 +38520,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A183" s="6">
         <v>182</v>
       </c>
@@ -38476,7 +38567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A184" s="6">
         <v>183</v>
       </c>
@@ -38523,7 +38614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A185" s="6">
         <v>184</v>
       </c>
@@ -38570,7 +38661,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A186" s="6">
         <v>185</v>
       </c>
@@ -38617,7 +38708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A187" s="6">
         <v>186</v>
       </c>
@@ -38664,7 +38755,7 @@
         <v>252000</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A188" s="6">
         <v>187</v>
       </c>
@@ -38711,7 +38802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A189" s="6">
         <v>188</v>
       </c>
@@ -38758,7 +38849,7 @@
         <v>280000</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A190" s="6">
         <v>189</v>
       </c>
@@ -38805,7 +38896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A191" s="6">
         <v>190</v>
       </c>
@@ -38852,7 +38943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A192" s="6">
         <v>191</v>
       </c>
@@ -38899,7 +38990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A193" s="6">
         <v>192</v>
       </c>
@@ -38946,7 +39037,7 @@
         <v>264000</v>
       </c>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A194" s="6">
         <v>193</v>
       </c>
@@ -38993,7 +39084,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A195" s="6">
         <v>194</v>
       </c>
@@ -39040,7 +39131,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A196" s="6">
         <v>195</v>
       </c>
@@ -39087,7 +39178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A197" s="6">
         <v>196</v>
       </c>
@@ -39134,7 +39225,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A198" s="6">
         <v>197</v>
       </c>
@@ -39181,7 +39272,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A199" s="6">
         <v>198</v>
       </c>
@@ -39228,7 +39319,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A200" s="6">
         <v>199</v>
       </c>
@@ -39275,7 +39366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A201" s="6">
         <v>200</v>
       </c>
@@ -39322,7 +39413,7 @@
         <v>265000</v>
       </c>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A202" s="6">
         <v>201</v>
       </c>
@@ -39369,7 +39460,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A203" s="6">
         <v>202</v>
       </c>
@@ -39416,7 +39507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A204" s="6">
         <v>203</v>
       </c>
@@ -39463,7 +39554,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A205" s="6">
         <v>204</v>
       </c>
@@ -39510,7 +39601,7 @@
         <v>260000</v>
       </c>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A206" s="6">
         <v>205</v>
       </c>
@@ -39557,7 +39648,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A207" s="6">
         <v>206</v>
       </c>
@@ -39604,7 +39695,7 @@
         <v>250000</v>
       </c>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A208" s="6">
         <v>207</v>
       </c>
@@ -39651,7 +39742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A209" s="6">
         <v>208</v>
       </c>
@@ -39698,7 +39789,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A210" s="6">
         <v>209</v>
       </c>
@@ -39745,7 +39836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A211" s="6">
         <v>210</v>
       </c>
@@ -39792,7 +39883,7 @@
         <v>216000</v>
       </c>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A212" s="6">
         <v>211</v>
       </c>
@@ -39839,7 +39930,7 @@
         <v>400000</v>
       </c>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A213" s="6">
         <v>212</v>
       </c>
@@ -39886,7 +39977,7 @@
         <v>275000</v>
       </c>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A214" s="6">
         <v>213</v>
       </c>
@@ -39933,7 +40024,7 @@
         <v>295000</v>
       </c>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A215" s="6">
         <v>214</v>
       </c>
@@ -39980,7 +40071,7 @@
         <v>204000</v>
       </c>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A216" s="6">
         <v>215</v>
       </c>
@@ -40038,24 +40129,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CA1432C-5E0A-4E92-8CB2-732177D70D2B}">
   <dimension ref="A1:M57"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -40066,7 +40157,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
@@ -40083,7 +40174,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
@@ -40103,7 +40194,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>31</v>
       </c>
@@ -40111,17 +40202,17 @@
         <v>215</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="J26" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
@@ -40129,7 +40220,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>30</v>
       </c>
@@ -40149,7 +40240,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>19</v>
       </c>
@@ -40175,7 +40266,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>24</v>
       </c>
@@ -40201,7 +40292,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>31</v>
       </c>
@@ -40227,7 +40318,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="J32" s="3" t="s">
         <v>31</v>
       </c>
@@ -40241,18 +40332,18 @@
         <v>215</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>37</v>
       </c>
       <c r="J50" s="4"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="J51" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>32</v>
       </c>
@@ -40260,7 +40351,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>30</v>
       </c>
@@ -40280,7 +40371,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>27</v>
       </c>
@@ -40300,7 +40391,7 @@
         <v>236591.66666666666</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>16</v>
       </c>
@@ -40320,7 +40411,7 @@
         <v>148315.78947368421</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>18</v>
       </c>
@@ -40340,7 +40431,7 @@
         <v>197586.04651162791</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>31</v>
       </c>
@@ -40363,12 +40454,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DD91E2A-760D-4ED4-BC23-C14C12431369}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="8.7265625" style="10"/>
+    <col min="1" max="16384" width="8.77734375" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="35" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:19" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A1" s="8" t="s">
         <v>40</v>
       </c>
@@ -40391,7 +40482,7 @@
       <c r="R1" s="9"/>
       <c r="S1" s="9"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>

</xml_diff>